<commit_message>
Actualizar maestros de proveedores (7 nuevos, 1 reclasificado)
Sincronización con nueva exportación del sistema contable (5023 registros):
- 7 proveedores nuevos agregados.
- 1 proveedor con nombre y gasto/rubro actualizados: CUIT 55000004382,
  "CMS HASCHE SINGLE" -> "LANGNESE HONGIG GMBH & CO KG", gasto/rubro
  (6,5) -> (0,0).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDWMgb28y7wbJrgi8xhXfb
</commit_message>
<xml_diff>
--- a/cuit_nombre.xlsx
+++ b/cuit_nombre.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5006"/>
+  <dimension ref="A1:B5013"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -10012,7 +10012,6 @@
       </c>
     </row>
     <row r="798">
-      <c r="A798" t="inlineStr"/>
       <c r="B798" t="inlineStr">
         <is>
           <t>ANTONIOLLI HOTEIS E TURISMO SA</t>
@@ -10020,7 +10019,6 @@
       </c>
     </row>
     <row r="799">
-      <c r="A799" t="inlineStr"/>
       <c r="B799" t="inlineStr">
         <is>
           <t>APPLE SUL RESTAURANTE</t>
@@ -10028,7 +10026,6 @@
       </c>
     </row>
     <row r="800">
-      <c r="A800" t="inlineStr"/>
       <c r="B800" t="inlineStr">
         <is>
           <t>HOTEL BAVARIA</t>
@@ -10036,7 +10033,6 @@
       </c>
     </row>
     <row r="801">
-      <c r="A801" t="inlineStr"/>
       <c r="B801" t="inlineStr">
         <is>
           <t>AEROPORTO INTERN. SAO PAULO</t>
@@ -10056,7 +10052,6 @@
       </c>
     </row>
     <row r="803">
-      <c r="A803" t="inlineStr"/>
       <c r="B803" t="inlineStr">
         <is>
           <t>WMS SUPERMERCARDOS</t>
@@ -10076,7 +10071,6 @@
       </c>
     </row>
     <row r="805">
-      <c r="A805" t="inlineStr"/>
       <c r="B805" t="inlineStr">
         <is>
           <t>LLFX COMERCIO DE ALIM</t>
@@ -10084,7 +10078,6 @@
       </c>
     </row>
     <row r="806">
-      <c r="A806" t="inlineStr"/>
       <c r="B806" t="inlineStr">
         <is>
           <t>SNOWLAND</t>
@@ -10740,7 +10733,6 @@
       </c>
     </row>
     <row r="861">
-      <c r="A861" t="inlineStr"/>
       <c r="B861" t="inlineStr">
         <is>
           <t>OMNI HOTELS</t>
@@ -10748,7 +10740,6 @@
       </c>
     </row>
     <row r="862">
-      <c r="A862" t="inlineStr"/>
       <c r="B862" t="inlineStr">
         <is>
           <t>WELCOME SAN ANTONIO</t>
@@ -16768,7 +16759,6 @@
       </c>
     </row>
     <row r="1364">
-      <c r="A1364" t="inlineStr"/>
       <c r="B1364" t="inlineStr">
         <is>
           <t>SYSTEM AMERICAN CARGO</t>
@@ -29520,7 +29510,6 @@
       </c>
     </row>
     <row r="2427">
-      <c r="A2427" t="inlineStr"/>
       <c r="B2427" t="inlineStr">
         <is>
           <t>FEDERACI”N DE COOPERATIVAS</t>
@@ -32060,7 +32049,6 @@
       </c>
     </row>
     <row r="2639">
-      <c r="A2639" t="inlineStr"/>
       <c r="B2639" t="inlineStr">
         <is>
           <t>BANCO DE INVERCION Y COMER. EX</t>
@@ -32583,10 +32571,7 @@
         </is>
       </c>
     </row>
-    <row r="2683">
-      <c r="A2683" t="inlineStr"/>
-      <c r="B2683" t="inlineStr"/>
-    </row>
+    <row r="2683"/>
     <row r="2684">
       <c r="A2684" t="inlineStr">
         <is>
@@ -33823,10 +33808,7 @@
         </is>
       </c>
     </row>
-    <row r="2787">
-      <c r="A2787" t="inlineStr"/>
-      <c r="B2787" t="inlineStr"/>
-    </row>
+    <row r="2787"/>
     <row r="2788">
       <c r="A2788" t="inlineStr">
         <is>
@@ -34103,10 +34085,7 @@
         </is>
       </c>
     </row>
-    <row r="2811">
-      <c r="A2811" t="inlineStr"/>
-      <c r="B2811" t="inlineStr"/>
-    </row>
+    <row r="2811"/>
     <row r="2812">
       <c r="A2812" t="inlineStr">
         <is>
@@ -42460,7 +42439,6 @@
       </c>
     </row>
     <row r="3508">
-      <c r="A3508" t="inlineStr"/>
       <c r="B3508" t="inlineStr">
         <is>
           <t>ESTACION DE SERV. YPF SUNCHALE</t>
@@ -46411,7 +46389,7 @@
       </c>
       <c r="B3837" t="inlineStr">
         <is>
-          <t>CMS HASCHE SINGLE</t>
+          <t>LANGNESE HONGIG GMBH &amp; CO KG</t>
         </is>
       </c>
     </row>
@@ -49452,7 +49430,6 @@
       </c>
     </row>
     <row r="4091">
-      <c r="A4091" t="inlineStr"/>
       <c r="B4091" t="inlineStr">
         <is>
           <t>VERSALLI GUSTAVO</t>
@@ -52352,7 +52329,6 @@
       </c>
     </row>
     <row r="4333">
-      <c r="A4333" t="inlineStr"/>
       <c r="B4333" t="inlineStr">
         <is>
           <t xml:space="preserve"> DARRECHON ARIEL EDGARDO</t>
@@ -52527,10 +52503,7 @@
         </is>
       </c>
     </row>
-    <row r="4348">
-      <c r="A4348" t="inlineStr"/>
-      <c r="B4348" t="inlineStr"/>
-    </row>
+    <row r="4348"/>
     <row r="4349">
       <c r="A4349" t="inlineStr">
         <is>
@@ -52567,10 +52540,7 @@
         </is>
       </c>
     </row>
-    <row r="4352">
-      <c r="A4352" t="inlineStr"/>
-      <c r="B4352" t="inlineStr"/>
-    </row>
+    <row r="4352"/>
     <row r="4353">
       <c r="A4353" t="inlineStr">
         <is>
@@ -52823,10 +52793,7 @@
         </is>
       </c>
     </row>
-    <row r="4374">
-      <c r="A4374" t="inlineStr"/>
-      <c r="B4374" t="inlineStr"/>
-    </row>
+    <row r="4374"/>
     <row r="4375">
       <c r="A4375" t="inlineStr">
         <is>
@@ -52935,10 +52902,7 @@
         </is>
       </c>
     </row>
-    <row r="4384">
-      <c r="A4384" t="inlineStr"/>
-      <c r="B4384" t="inlineStr"/>
-    </row>
+    <row r="4384"/>
     <row r="4385">
       <c r="A4385" t="inlineStr">
         <is>
@@ -56251,10 +56215,7 @@
         </is>
       </c>
     </row>
-    <row r="4661">
-      <c r="A4661" t="inlineStr"/>
-      <c r="B4661" t="inlineStr"/>
-    </row>
+    <row r="4661"/>
     <row r="4662">
       <c r="A4662" t="inlineStr">
         <is>
@@ -59099,10 +59060,7 @@
         </is>
       </c>
     </row>
-    <row r="4899">
-      <c r="A4899" t="inlineStr"/>
-      <c r="B4899" t="inlineStr"/>
-    </row>
+    <row r="4899"/>
     <row r="4900">
       <c r="A4900" t="inlineStr">
         <is>
@@ -59415,10 +59373,7 @@
         </is>
       </c>
     </row>
-    <row r="4926">
-      <c r="A4926" t="inlineStr"/>
-      <c r="B4926" t="inlineStr"/>
-    </row>
+    <row r="4926"/>
     <row r="4927">
       <c r="A4927" t="inlineStr">
         <is>
@@ -59431,10 +59386,7 @@
         </is>
       </c>
     </row>
-    <row r="4928">
-      <c r="A4928" t="inlineStr"/>
-      <c r="B4928" t="inlineStr"/>
-    </row>
+    <row r="4928"/>
     <row r="4929">
       <c r="A4929" t="inlineStr">
         <is>
@@ -59459,10 +59411,7 @@
         </is>
       </c>
     </row>
-    <row r="4931">
-      <c r="A4931" t="inlineStr"/>
-      <c r="B4931" t="inlineStr"/>
-    </row>
+    <row r="4931"/>
     <row r="4932">
       <c r="A4932" t="inlineStr">
         <is>
@@ -60028,7 +59977,6 @@
       </c>
     </row>
     <row r="4979">
-      <c r="A4979" t="inlineStr"/>
       <c r="B4979" t="inlineStr">
         <is>
           <t>SCHONFELD MATIAS NAHUEL</t>
@@ -60107,10 +60055,7 @@
         </is>
       </c>
     </row>
-    <row r="4986">
-      <c r="A4986" t="inlineStr"/>
-      <c r="B4986" t="inlineStr"/>
-    </row>
+    <row r="4986"/>
     <row r="4987">
       <c r="A4987" t="inlineStr">
         <is>
@@ -60348,6 +60293,90 @@
       <c r="B5006" t="inlineStr">
         <is>
           <t>PATAT SRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5007">
+      <c r="A5007" t="inlineStr">
+        <is>
+          <t>20206736276</t>
+        </is>
+      </c>
+      <c r="B5007" t="inlineStr">
+        <is>
+          <t>ALCIBAR CRISTIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5008">
+      <c r="A5008" t="inlineStr">
+        <is>
+          <t>20285632448</t>
+        </is>
+      </c>
+      <c r="B5008" t="inlineStr">
+        <is>
+          <t>BROGNO JUAN AUGUSTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5009">
+      <c r="A5009" t="inlineStr">
+        <is>
+          <t>20131149248</t>
+        </is>
+      </c>
+      <c r="B5009" t="inlineStr">
+        <is>
+          <t>QUINTANA JULIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5010">
+      <c r="A5010" t="inlineStr">
+        <is>
+          <t>20164301797</t>
+        </is>
+      </c>
+      <c r="B5010" t="inlineStr">
+        <is>
+          <t>MURILLO RUBEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5011">
+      <c r="A5011" t="inlineStr">
+        <is>
+          <t>23167820719</t>
+        </is>
+      </c>
+      <c r="B5011" t="inlineStr">
+        <is>
+          <t>VARGAS JUAN JOSE  (PADRE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5012">
+      <c r="A5012" t="inlineStr">
+        <is>
+          <t>20104183671</t>
+        </is>
+      </c>
+      <c r="B5012" t="inlineStr">
+        <is>
+          <t>ROMERO HORACIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5013">
+      <c r="A5013" t="inlineStr">
+        <is>
+          <t>24284239918</t>
+        </is>
+      </c>
+      <c r="B5013" t="inlineStr">
+        <is>
+          <t>AGUIRRE SABRINA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar maestros de proveedores (10 nuevos, 2 reclasificados)
Sincronización con nueva exportación del sistema contable (5027 registros):
- 10 proveedores nuevos agregados.
- 2 reclasificados a gasto/rubro (0,0): LORA SERGIO DANIEL y PISTARINI
  MARCELO FABIAN (antes g4,r6).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDWMgb28y7wbJrgi8xhXfb
</commit_message>
<xml_diff>
--- a/cuit_nombre.xlsx
+++ b/cuit_nombre.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5013"/>
+  <dimension ref="A1:B5023"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -60380,6 +60380,126 @@
         </is>
       </c>
     </row>
+    <row r="5014">
+      <c r="A5014" t="inlineStr">
+        <is>
+          <t>30714439304</t>
+        </is>
+      </c>
+      <c r="B5014" t="inlineStr">
+        <is>
+          <t>MODOC SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5015">
+      <c r="A5015" t="inlineStr">
+        <is>
+          <t>20373443515</t>
+        </is>
+      </c>
+      <c r="B5015" t="inlineStr">
+        <is>
+          <t>CATIBIELA MARTIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5016">
+      <c r="A5016" t="inlineStr">
+        <is>
+          <t>23389167649</t>
+        </is>
+      </c>
+      <c r="B5016" t="inlineStr">
+        <is>
+          <t>MOISES DOMINGUEZ TOMAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5017">
+      <c r="A5017" t="inlineStr">
+        <is>
+          <t>20124747318</t>
+        </is>
+      </c>
+      <c r="B5017" t="inlineStr">
+        <is>
+          <t>KUHLMANN MARIO ALBERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5018">
+      <c r="A5018" t="inlineStr">
+        <is>
+          <t>20332711432</t>
+        </is>
+      </c>
+      <c r="B5018" t="inlineStr">
+        <is>
+          <t>PUIG PABLO FEDERICO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5019">
+      <c r="A5019" t="inlineStr">
+        <is>
+          <t>20267967254</t>
+        </is>
+      </c>
+      <c r="B5019" t="inlineStr">
+        <is>
+          <t>ECHEVESTE KEVIN EMANUEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5020">
+      <c r="A5020" t="inlineStr">
+        <is>
+          <t>20224756020</t>
+        </is>
+      </c>
+      <c r="B5020" t="inlineStr">
+        <is>
+          <t>VAN DER HORST EDUARDO ANDRES</t>
+        </is>
+      </c>
+    </row>
+    <row r="5021">
+      <c r="A5021" t="inlineStr">
+        <is>
+          <t>20217048541</t>
+        </is>
+      </c>
+      <c r="B5021" t="inlineStr">
+        <is>
+          <t>YANACONE MARIO FABIAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5022">
+      <c r="A5022" t="inlineStr">
+        <is>
+          <t>20120633210</t>
+        </is>
+      </c>
+      <c r="B5022" t="inlineStr">
+        <is>
+          <t>AGUERRALDE CESAR ALBERTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5023">
+      <c r="A5023" t="inlineStr">
+        <is>
+          <t>30586347760</t>
+        </is>
+      </c>
+      <c r="B5023" t="inlineStr">
+        <is>
+          <t>ENVAPLAST SRL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar maestros de proveedores (10 nuevos, 1 reclasificado)
Sincronización con nueva exportación del sistema contable (5029 registros):
- 10 proveedores nuevos agregados.
- 1 reclasificado a gasto/rubro (0,0): GAMBERO RAUL EMILIO (antes g4,r6).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDWMgb28y7wbJrgi8xhXfb
</commit_message>
<xml_diff>
--- a/cuit_nombre.xlsx
+++ b/cuit_nombre.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5023"/>
+  <dimension ref="A1:B5033"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -60500,6 +60500,126 @@
         </is>
       </c>
     </row>
+    <row r="5024">
+      <c r="A5024" t="inlineStr">
+        <is>
+          <t>30719266017</t>
+        </is>
+      </c>
+      <c r="B5024" t="inlineStr">
+        <is>
+          <t>CARDAL SAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5025">
+      <c r="A5025" t="inlineStr">
+        <is>
+          <t>20459484915</t>
+        </is>
+      </c>
+      <c r="B5025" t="inlineStr">
+        <is>
+          <t>DIAZ ALEXANDER DYLAN NATAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="5026">
+      <c r="A5026" t="inlineStr">
+        <is>
+          <t>20180846825</t>
+        </is>
+      </c>
+      <c r="B5026" t="inlineStr">
+        <is>
+          <t>PEREZ GUSTAVO ANIBAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5027">
+      <c r="A5027" t="inlineStr">
+        <is>
+          <t>20164000495</t>
+        </is>
+      </c>
+      <c r="B5027" t="inlineStr">
+        <is>
+          <t>GARCIA DIEGO A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5028">
+      <c r="A5028" t="inlineStr">
+        <is>
+          <t>30657282207</t>
+        </is>
+      </c>
+      <c r="B5028" t="inlineStr">
+        <is>
+          <t>METALURGICA HERMANN SRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5029">
+      <c r="A5029" t="inlineStr">
+        <is>
+          <t>30516150641</t>
+        </is>
+      </c>
+      <c r="B5029" t="inlineStr">
+        <is>
+          <t>VOLVO TRUCKS Y BUSES ARGENTINA SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5030">
+      <c r="A5030" t="inlineStr">
+        <is>
+          <t>30711824975</t>
+        </is>
+      </c>
+      <c r="B5030" t="inlineStr">
+        <is>
+          <t>ZAPPA JUAN PABLO Y ZAPPA CARLOS SH</t>
+        </is>
+      </c>
+    </row>
+    <row r="5031">
+      <c r="A5031" t="inlineStr">
+        <is>
+          <t>20223875646</t>
+        </is>
+      </c>
+      <c r="B5031" t="inlineStr">
+        <is>
+          <t>LOPEZ DE SABANDO FERNANDO CESAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5032">
+      <c r="A5032" t="inlineStr">
+        <is>
+          <t>20395783832</t>
+        </is>
+      </c>
+      <c r="B5032" t="inlineStr">
+        <is>
+          <t>SCHONFELD MATIAS NAHUEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5033">
+      <c r="A5033" t="inlineStr">
+        <is>
+          <t>27223189011</t>
+        </is>
+      </c>
+      <c r="B5033" t="inlineStr">
+        <is>
+          <t>ALZAMORA NORA ALEJANDRA</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>